<commit_message>
Add Order Grouping Sorter and sync local warehouse work to GitHub.
Brings this PC in line with origin/main: sorter app, taxonomy pick-lists, packing/shipping updates, and related rules — excluding live DBs, secrets, debug logs, and run I/O.
</commit_message>
<xml_diff>
--- a/Order Grouping for Packing List.xlsx
+++ b/Order Grouping for Packing List.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Warehouse Operations System\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Areeb Work\Warehouse Operations System\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CF1BA81-D9CE-49E1-BFFB-2DA0DBF2295C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{822F9C74-0DDF-4EDD-A685-D8B36178F222}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Graph" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="447" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="447" uniqueCount="160">
   <si>
     <t>resend</t>
   </si>
@@ -155,9 +155,6 @@
   </si>
   <si>
     <t>shipping-service</t>
-  </si>
-  <si>
-    <t>produt-finish</t>
   </si>
   <si>
     <t>today-plain-all_channels-x-prime-dtf-readymade-x</t>
@@ -697,7 +694,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -774,17 +771,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -792,13 +780,10 @@
     <xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1082,80 +1067,80 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AY42"/>
-  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.90625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="1.90625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.7265625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="3" style="29" customWidth="1"/>
-    <col min="5" max="5" width="7.36328125" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.26953125" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.54296875" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="3.81640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="3.81640625" style="29" customWidth="1"/>
-    <col min="10" max="10" width="20.54296875" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="1.90625" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="24.08984375" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="1.90625" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="15.81640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="1.90625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="1.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="3" style="1" customWidth="1"/>
+    <col min="5" max="5" width="7.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="3.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="3.77734375" style="1" customWidth="1"/>
+    <col min="10" max="10" width="20.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="1.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="24.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="1.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="1.88671875" style="1" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="15" style="1" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="1.90625" style="1" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="15.08984375" style="1" customWidth="1"/>
-    <col min="19" max="19" width="1.90625" style="1" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="1.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="15.109375" style="1" customWidth="1"/>
+    <col min="19" max="19" width="1.88671875" style="1" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="14" style="1" customWidth="1"/>
-    <col min="21" max="21" width="1.90625" style="1" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="17.54296875" style="1" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="1.90625" style="1" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="1.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="17.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="1.88671875" style="1" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="9" style="1" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="1.90625" style="1" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="12.81640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="1.90625" style="1" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="18.6328125" style="1" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="1.90625" style="1" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="13.36328125" style="1" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="1.90625" style="1" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="12.26953125" style="1" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="1.90625" style="1" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="8.7265625" style="1" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="2.81640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="1.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="12.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="1.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="18.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="1.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="13.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="1.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="12.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="1.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="8.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="2.77734375" style="1" bestFit="1" customWidth="1"/>
     <col min="36" max="36" width="12" style="1" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="2.81640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="12.26953125" style="1" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="2.81640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="2.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="12.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="2.77734375" style="1" bestFit="1" customWidth="1"/>
     <col min="40" max="40" width="11" style="1" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="2.81640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="8.7265625" style="1" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="2.81640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="8.7265625" style="1" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="2.81640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="8.7265625" style="1" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="2.81640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="5.26953125" style="1" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="5.453125" style="1" bestFit="1" customWidth="1"/>
-    <col min="50" max="50" width="21.26953125" style="1" bestFit="1" customWidth="1"/>
-    <col min="51" max="51" width="52.1796875" style="1" bestFit="1" customWidth="1"/>
-    <col min="52" max="16384" width="8.90625" style="1"/>
+    <col min="41" max="41" width="2.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="8.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="2.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="8.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="2.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="8.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="2.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="5.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="5.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="21.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="51" max="51" width="52.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="52" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:51" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:51" x14ac:dyDescent="0.3">
       <c r="A1" s="12" t="s">
-        <v>48</v>
-      </c>
-      <c r="B1" s="27"/>
+        <v>47</v>
+      </c>
+      <c r="B1" s="26"/>
       <c r="C1" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="D1" s="28"/>
-      <c r="E1" s="26" t="s">
-        <v>50</v>
-      </c>
-      <c r="F1" s="26"/>
-      <c r="G1" s="26"/>
-      <c r="H1" s="26"/>
-      <c r="I1" s="28"/>
+      <c r="D1" s="23"/>
+      <c r="E1" s="29" t="s">
+        <v>49</v>
+      </c>
+      <c r="F1" s="29"/>
+      <c r="G1" s="29"/>
+      <c r="H1" s="29"/>
+      <c r="I1" s="23"/>
       <c r="J1" s="2" t="s">
-        <v>43</v>
+        <v>98</v>
       </c>
       <c r="L1" s="2" t="s">
         <v>38</v>
@@ -1173,7 +1158,7 @@
         <v>22</v>
       </c>
       <c r="V1" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="X1" s="2" t="s">
         <v>25</v>
@@ -1197,7 +1182,7 @@
         <v>4</v>
       </c>
       <c r="AL1" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="AN1" s="2" t="s">
         <v>7</v>
@@ -1212,99 +1197,99 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:51" s="29" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="30" t="s">
+    <row r="2" spans="1:51" x14ac:dyDescent="0.3">
+      <c r="A2" s="27" t="s">
+        <v>157</v>
+      </c>
+      <c r="B2" s="26"/>
+      <c r="C2" s="27" t="s">
+        <v>157</v>
+      </c>
+      <c r="D2" s="26"/>
+      <c r="E2" s="30" t="s">
+        <v>95</v>
+      </c>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
+      <c r="H2" s="28"/>
+      <c r="I2" s="23"/>
+      <c r="J2" s="28" t="s">
         <v>158</v>
       </c>
-      <c r="B2" s="27"/>
-      <c r="C2" s="30" t="s">
-        <v>158</v>
-      </c>
-      <c r="D2" s="27"/>
-      <c r="E2" s="32" t="s">
-        <v>96</v>
-      </c>
-      <c r="F2" s="32"/>
-      <c r="G2" s="32"/>
-      <c r="H2" s="31"/>
-      <c r="I2" s="28"/>
-      <c r="J2" s="31" t="s">
+      <c r="K2" s="23"/>
+      <c r="L2" s="28" t="s">
         <v>159</v>
       </c>
-      <c r="K2" s="28"/>
-      <c r="L2" s="31" t="s">
-        <v>160</v>
-      </c>
-      <c r="M2" s="28"/>
-      <c r="N2" s="31" t="s">
-        <v>96</v>
-      </c>
-      <c r="O2" s="28"/>
-      <c r="P2" s="31" t="s">
-        <v>158</v>
-      </c>
-      <c r="Q2" s="28"/>
-      <c r="R2" s="31" t="s">
-        <v>75</v>
-      </c>
-      <c r="S2" s="28"/>
-      <c r="T2" s="31" t="s">
-        <v>75</v>
-      </c>
-      <c r="U2" s="28"/>
-      <c r="V2" s="31" t="s">
-        <v>75</v>
-      </c>
-      <c r="W2" s="28"/>
-      <c r="X2" s="31" t="s">
-        <v>75</v>
-      </c>
-      <c r="Y2" s="28"/>
-      <c r="Z2" s="31" t="s">
-        <v>75</v>
-      </c>
-      <c r="AA2" s="28"/>
-      <c r="AB2" s="31" t="s">
-        <v>75</v>
-      </c>
-      <c r="AC2" s="28"/>
-      <c r="AD2" s="31" t="s">
-        <v>75</v>
-      </c>
-      <c r="AE2" s="28"/>
-      <c r="AF2" s="31" t="s">
-        <v>75</v>
-      </c>
-      <c r="AG2" s="28"/>
-      <c r="AH2" s="31" t="s">
-        <v>75</v>
-      </c>
-      <c r="AI2" s="28"/>
-      <c r="AJ2" s="31" t="s">
-        <v>75</v>
-      </c>
-      <c r="AK2" s="28"/>
-      <c r="AL2" s="31" t="s">
-        <v>75</v>
-      </c>
-      <c r="AM2" s="28"/>
-      <c r="AN2" s="31" t="s">
-        <v>75</v>
-      </c>
-      <c r="AO2" s="28"/>
-      <c r="AP2" s="31" t="s">
-        <v>75</v>
-      </c>
-      <c r="AQ2" s="28"/>
-      <c r="AR2" s="31" t="s">
-        <v>75</v>
-      </c>
-      <c r="AS2" s="28"/>
-      <c r="AT2" s="31" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="3" spans="1:51" x14ac:dyDescent="0.35">
+      <c r="M2" s="23"/>
+      <c r="N2" s="28" t="s">
+        <v>95</v>
+      </c>
+      <c r="O2" s="23"/>
+      <c r="P2" s="28" t="s">
+        <v>157</v>
+      </c>
+      <c r="Q2" s="23"/>
+      <c r="R2" s="28" t="s">
+        <v>74</v>
+      </c>
+      <c r="S2" s="23"/>
+      <c r="T2" s="28" t="s">
+        <v>74</v>
+      </c>
+      <c r="U2" s="23"/>
+      <c r="V2" s="28" t="s">
+        <v>74</v>
+      </c>
+      <c r="W2" s="23"/>
+      <c r="X2" s="28" t="s">
+        <v>74</v>
+      </c>
+      <c r="Y2" s="23"/>
+      <c r="Z2" s="28" t="s">
+        <v>74</v>
+      </c>
+      <c r="AA2" s="23"/>
+      <c r="AB2" s="28" t="s">
+        <v>74</v>
+      </c>
+      <c r="AC2" s="23"/>
+      <c r="AD2" s="28" t="s">
+        <v>74</v>
+      </c>
+      <c r="AE2" s="23"/>
+      <c r="AF2" s="28" t="s">
+        <v>74</v>
+      </c>
+      <c r="AG2" s="23"/>
+      <c r="AH2" s="28" t="s">
+        <v>74</v>
+      </c>
+      <c r="AI2" s="23"/>
+      <c r="AJ2" s="28" t="s">
+        <v>74</v>
+      </c>
+      <c r="AK2" s="23"/>
+      <c r="AL2" s="28" t="s">
+        <v>74</v>
+      </c>
+      <c r="AM2" s="23"/>
+      <c r="AN2" s="28" t="s">
+        <v>74</v>
+      </c>
+      <c r="AO2" s="23"/>
+      <c r="AP2" s="28" t="s">
+        <v>74</v>
+      </c>
+      <c r="AQ2" s="23"/>
+      <c r="AR2" s="28" t="s">
+        <v>74</v>
+      </c>
+      <c r="AS2" s="23"/>
+      <c r="AT2" s="28" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="3" spans="1:51" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
         <v>0</v>
       </c>
@@ -1312,19 +1297,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:51" x14ac:dyDescent="0.35">
-      <c r="A4" s="29"/>
-      <c r="B4" s="29"/>
-    </row>
-    <row r="5" spans="1:51" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:51" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B5" s="3">
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:51" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:51" x14ac:dyDescent="0.3">
       <c r="C7" s="3" t="s">
         <v>31</v>
       </c>
@@ -1335,13 +1316,13 @@
         <v>1</v>
       </c>
       <c r="L7" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="M7" s="3">
         <v>1</v>
       </c>
       <c r="N7" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="O7" s="3" t="s">
         <v>37</v>
@@ -1353,7 +1334,7 @@
         <v>1</v>
       </c>
       <c r="R7" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="S7" s="3" t="s">
         <v>37</v>
@@ -1365,55 +1346,55 @@
         <v>37</v>
       </c>
       <c r="V7" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="W7" s="3" t="s">
         <v>37</v>
       </c>
       <c r="X7" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="Y7" s="3" t="s">
         <v>37</v>
       </c>
       <c r="Z7" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="AA7" s="3" t="s">
         <v>37</v>
       </c>
       <c r="AB7" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="AC7" s="3">
         <v>1</v>
       </c>
       <c r="AD7" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="AE7" s="3">
         <v>1</v>
       </c>
       <c r="AF7" s="3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="AG7" s="3">
         <v>1</v>
       </c>
       <c r="AH7" s="3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AI7" s="3">
         <v>30</v>
       </c>
       <c r="AX7" s="9" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="AY7" s="11" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="8" spans="1:51" x14ac:dyDescent="0.35">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="8" spans="1:51" x14ac:dyDescent="0.3">
       <c r="P8" s="6" t="s">
         <v>23</v>
       </c>
@@ -1421,7 +1402,7 @@
         <v>1</v>
       </c>
       <c r="T8" s="6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="U8" s="6" t="s">
         <v>37</v>
@@ -1430,30 +1411,30 @@
         <v>5</v>
       </c>
       <c r="AJ8" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="AK8" s="3">
         <v>30</v>
       </c>
       <c r="AX8" s="10" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="AY8" s="11" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="9" spans="1:51" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:51" x14ac:dyDescent="0.3">
       <c r="AK9" s="3" t="s">
         <v>5</v>
       </c>
       <c r="AL9" s="3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AM9" s="3">
         <v>30</v>
       </c>
     </row>
-    <row r="10" spans="1:51" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:51" x14ac:dyDescent="0.3">
       <c r="E10" s="13"/>
       <c r="F10" s="14" t="s">
         <v>34</v>
@@ -1462,18 +1443,17 @@
         <v>500</v>
       </c>
       <c r="H10" s="25"/>
-      <c r="I10" s="33"/>
       <c r="AM10" s="3" t="s">
         <v>5</v>
       </c>
       <c r="AN10" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AO10" s="3">
         <v>30</v>
       </c>
     </row>
-    <row r="11" spans="1:51" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:51" x14ac:dyDescent="0.3">
       <c r="E11" s="16" t="s">
         <v>28</v>
       </c>
@@ -1486,18 +1466,17 @@
       <c r="H11" s="17">
         <v>300</v>
       </c>
-      <c r="I11" s="33"/>
       <c r="AO11" s="3" t="s">
         <v>5</v>
       </c>
       <c r="AP11" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="AQ11" s="3">
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="1:51" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:51" x14ac:dyDescent="0.3">
       <c r="E12" s="18"/>
       <c r="G12" s="3" t="s">
         <v>35</v>
@@ -1505,33 +1484,32 @@
       <c r="H12" s="17">
         <v>200</v>
       </c>
-      <c r="I12" s="33"/>
       <c r="AQ12" s="3" t="s">
         <v>5</v>
       </c>
       <c r="AR12" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AS12" s="3">
         <v>30</v>
       </c>
     </row>
-    <row r="13" spans="1:51" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:51" x14ac:dyDescent="0.3">
       <c r="E13" s="18"/>
       <c r="G13" s="23"/>
       <c r="H13" s="24"/>
-      <c r="I13" s="34"/>
+      <c r="I13" s="23"/>
       <c r="AS13" s="3" t="s">
         <v>5</v>
       </c>
       <c r="AT13" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="AU13" s="3">
         <v>30</v>
       </c>
     </row>
-    <row r="14" spans="1:51" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:51" x14ac:dyDescent="0.3">
       <c r="E14" s="16" t="s">
         <v>29</v>
       </c>
@@ -1544,7 +1522,6 @@
       <c r="H14" s="17">
         <v>100</v>
       </c>
-      <c r="I14" s="33"/>
       <c r="AU14" s="3" t="s">
         <v>5</v>
       </c>
@@ -1555,7 +1532,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:51" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:51" x14ac:dyDescent="0.3">
       <c r="E15" s="18"/>
       <c r="G15" s="3" t="s">
         <v>35</v>
@@ -1563,7 +1540,6 @@
       <c r="H15" s="17">
         <v>400</v>
       </c>
-      <c r="I15" s="33"/>
       <c r="AV15" s="3" t="s">
         <v>11</v>
       </c>
@@ -1571,11 +1547,11 @@
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:51" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:51" x14ac:dyDescent="0.3">
       <c r="E16" s="18"/>
       <c r="G16" s="23"/>
       <c r="H16" s="24"/>
-      <c r="I16" s="34"/>
+      <c r="I16" s="23"/>
       <c r="AV16" s="3" t="s">
         <v>12</v>
       </c>
@@ -1583,7 +1559,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="5:49" x14ac:dyDescent="0.35">
+    <row r="17" spans="5:49" x14ac:dyDescent="0.3">
       <c r="E17" s="16" t="s">
         <v>30</v>
       </c>
@@ -1596,9 +1572,8 @@
       <c r="H17" s="17">
         <v>100</v>
       </c>
-      <c r="I17" s="33"/>
-    </row>
-    <row r="18" spans="5:49" x14ac:dyDescent="0.35">
+    </row>
+    <row r="18" spans="5:49" x14ac:dyDescent="0.3">
       <c r="E18" s="19"/>
       <c r="F18" s="20"/>
       <c r="G18" s="21" t="s">
@@ -1607,9 +1582,8 @@
       <c r="H18" s="22">
         <v>400</v>
       </c>
-      <c r="I18" s="33"/>
-    </row>
-    <row r="21" spans="5:49" x14ac:dyDescent="0.35">
+    </row>
+    <row r="21" spans="5:49" x14ac:dyDescent="0.3">
       <c r="J21" s="4" t="s">
         <v>17</v>
       </c>
@@ -1623,7 +1597,7 @@
         <v>1</v>
       </c>
       <c r="N21" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="O21" s="4">
         <v>0</v>
@@ -1635,7 +1609,7 @@
         <v>1</v>
       </c>
       <c r="R21" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="S21" s="4">
         <v>1</v>
@@ -1647,19 +1621,19 @@
         <v>1</v>
       </c>
       <c r="V21" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="W21" s="4" t="s">
         <v>37</v>
       </c>
       <c r="X21" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="Y21" s="4">
         <v>0</v>
       </c>
       <c r="Z21" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="AA21" s="4">
         <v>0</v>
@@ -1671,25 +1645,25 @@
         <v>1</v>
       </c>
       <c r="AD21" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="AE21" s="4" t="s">
         <v>37</v>
       </c>
       <c r="AF21" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="AG21" s="4">
         <v>0</v>
       </c>
       <c r="AH21" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AI21" s="4">
         <v>30</v>
       </c>
     </row>
-    <row r="22" spans="5:49" x14ac:dyDescent="0.35">
+    <row r="22" spans="5:49" x14ac:dyDescent="0.3">
       <c r="P22" s="6" t="s">
         <v>23</v>
       </c>
@@ -1697,7 +1671,7 @@
         <v>1</v>
       </c>
       <c r="T22" s="6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="U22" s="6">
         <v>1</v>
@@ -1706,68 +1680,68 @@
         <v>5</v>
       </c>
       <c r="AJ22" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="AK22" s="4">
         <v>30</v>
       </c>
     </row>
-    <row r="23" spans="5:49" x14ac:dyDescent="0.35">
+    <row r="23" spans="5:49" x14ac:dyDescent="0.3">
       <c r="AK23" s="4" t="s">
         <v>5</v>
       </c>
       <c r="AL23" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AM23" s="4">
         <v>30</v>
       </c>
     </row>
-    <row r="24" spans="5:49" x14ac:dyDescent="0.35">
+    <row r="24" spans="5:49" x14ac:dyDescent="0.3">
       <c r="AM24" s="4" t="s">
         <v>5</v>
       </c>
       <c r="AN24" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AO24" s="4">
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="5:49" x14ac:dyDescent="0.35">
+    <row r="25" spans="5:49" x14ac:dyDescent="0.3">
       <c r="AO25" s="4" t="s">
         <v>5</v>
       </c>
       <c r="AP25" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="AQ25" s="4">
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="5:49" x14ac:dyDescent="0.35">
+    <row r="26" spans="5:49" x14ac:dyDescent="0.3">
       <c r="AQ26" s="4" t="s">
         <v>5</v>
       </c>
       <c r="AR26" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AS26" s="4">
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="5:49" x14ac:dyDescent="0.35">
+    <row r="27" spans="5:49" x14ac:dyDescent="0.3">
       <c r="AS27" s="4" t="s">
         <v>5</v>
       </c>
       <c r="AT27" s="4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="AU27" s="4">
         <v>30</v>
       </c>
     </row>
-    <row r="28" spans="5:49" x14ac:dyDescent="0.35">
+    <row r="28" spans="5:49" x14ac:dyDescent="0.3">
       <c r="AU28" s="4" t="s">
         <v>5</v>
       </c>
@@ -1778,7 +1752,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="29" spans="5:49" x14ac:dyDescent="0.35">
+    <row r="29" spans="5:49" x14ac:dyDescent="0.3">
       <c r="AV29" s="4" t="s">
         <v>11</v>
       </c>
@@ -1786,7 +1760,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="30" spans="5:49" x14ac:dyDescent="0.35">
+    <row r="30" spans="5:49" x14ac:dyDescent="0.3">
       <c r="AV30" s="4" t="s">
         <v>12</v>
       </c>
@@ -1794,7 +1768,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="33" spans="28:50" x14ac:dyDescent="0.35">
+    <row r="33" spans="28:50" x14ac:dyDescent="0.3">
       <c r="AB33" s="7" t="s">
         <v>41</v>
       </c>
@@ -1802,92 +1776,92 @@
         <v>1</v>
       </c>
       <c r="AD33" s="7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="AE33" s="7">
         <v>1</v>
       </c>
       <c r="AF33" s="7" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="AG33" s="7">
         <v>0</v>
       </c>
       <c r="AH33" s="7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AI33" s="7">
         <v>30</v>
       </c>
     </row>
-    <row r="34" spans="28:50" x14ac:dyDescent="0.35">
+    <row r="34" spans="28:50" x14ac:dyDescent="0.3">
       <c r="AI34" s="7" t="s">
         <v>5</v>
       </c>
       <c r="AJ34" s="7" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="AK34" s="7">
         <v>30</v>
       </c>
     </row>
-    <row r="35" spans="28:50" x14ac:dyDescent="0.35">
+    <row r="35" spans="28:50" x14ac:dyDescent="0.3">
       <c r="AK35" s="7" t="s">
         <v>5</v>
       </c>
       <c r="AL35" s="7" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AM35" s="7">
         <v>30</v>
       </c>
     </row>
-    <row r="36" spans="28:50" x14ac:dyDescent="0.35">
+    <row r="36" spans="28:50" x14ac:dyDescent="0.3">
       <c r="AM36" s="7" t="s">
         <v>5</v>
       </c>
       <c r="AN36" s="7" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AO36" s="7">
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="28:50" x14ac:dyDescent="0.35">
+    <row r="37" spans="28:50" x14ac:dyDescent="0.3">
       <c r="AO37" s="7" t="s">
         <v>5</v>
       </c>
       <c r="AP37" s="7" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="AQ37" s="7">
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="28:50" x14ac:dyDescent="0.35">
+    <row r="38" spans="28:50" x14ac:dyDescent="0.3">
       <c r="AQ38" s="7" t="s">
         <v>5</v>
       </c>
       <c r="AR38" s="7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AS38" s="7">
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="28:50" x14ac:dyDescent="0.35">
+    <row r="39" spans="28:50" x14ac:dyDescent="0.3">
       <c r="AS39" s="7" t="s">
         <v>5</v>
       </c>
       <c r="AT39" s="7" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="AU39" s="7">
         <v>30</v>
       </c>
       <c r="AX39" s="8"/>
     </row>
-    <row r="40" spans="28:50" x14ac:dyDescent="0.35">
+    <row r="40" spans="28:50" x14ac:dyDescent="0.3">
       <c r="AU40" s="7" t="s">
         <v>5</v>
       </c>
@@ -1898,7 +1872,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="41" spans="28:50" x14ac:dyDescent="0.35">
+    <row r="41" spans="28:50" x14ac:dyDescent="0.3">
       <c r="AV41" s="7" t="s">
         <v>11</v>
       </c>
@@ -1906,7 +1880,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="42" spans="28:50" x14ac:dyDescent="0.35">
+    <row r="42" spans="28:50" x14ac:dyDescent="0.3">
       <c r="AV42" s="7" t="s">
         <v>12</v>
       </c>
@@ -1928,165 +1902,165 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF570E4C-BD7B-4204-8EC3-5BEA44270C66}">
   <dimension ref="A1:K41"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="23.26953125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="52.08984375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.26953125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.7265625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.36328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.90625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.7265625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.08984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="52.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.77734375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.44140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.77734375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="K1" s="2" t="s">
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A2" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="B2" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>82</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>83</v>
       </c>
       <c r="F2" s="1"/>
       <c r="G2" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H2" s="1"/>
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
       <c r="K2" s="1"/>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B3" s="7" t="s">
         <v>27</v>
       </c>
       <c r="C3" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="D3" s="1" t="s">
-        <v>87</v>
-      </c>
       <c r="E3" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F3" s="1"/>
       <c r="G3" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H3" s="1"/>
       <c r="I3" s="1"/>
       <c r="J3" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="K3" s="1"/>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
         <v>88</v>
-      </c>
-      <c r="K3" s="1"/>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A4" s="1" t="s">
-        <v>89</v>
       </c>
       <c r="B4" s="7" t="s">
         <v>36</v>
       </c>
       <c r="C4" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="E4" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="F4" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="E4" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="F4" s="1" t="s">
+      <c r="G4" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="H4" s="1" t="s">
         <v>92</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>93</v>
       </c>
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
       <c r="K4" s="1"/>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B5" s="7" t="s">
         <v>38</v>
       </c>
       <c r="C5" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="D5" s="1" t="s">
-        <v>96</v>
-      </c>
       <c r="E5" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F5" s="1"/>
       <c r="G5" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H5" s="1"/>
       <c r="I5" s="1"/>
       <c r="J5" s="1"/>
       <c r="K5" s="1"/>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B6" s="7" t="s">
         <v>42</v>
@@ -2095,48 +2069,48 @@
         <v>1</v>
       </c>
       <c r="D6" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="E6" s="1" t="s">
         <v>82</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>83</v>
       </c>
       <c r="F6" s="1"/>
       <c r="G6" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H6" s="1"/>
       <c r="I6" s="1"/>
       <c r="J6" s="1"/>
       <c r="K6" s="1"/>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="B7" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="C7" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="C7" s="1" t="s">
-        <v>100</v>
-      </c>
       <c r="D7" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F7" s="1"/>
       <c r="G7" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H7" s="1"/>
       <c r="I7" s="1"/>
       <c r="J7" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="K7" s="1"/>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>3</v>
       </c>
@@ -2144,86 +2118,86 @@
         <v>3</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D8" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="F8" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="E8" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>92</v>
-      </c>
       <c r="G8" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H8" s="1"/>
       <c r="I8" s="1"/>
       <c r="J8" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="K8" s="1"/>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B9" s="7" t="s">
         <v>4</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D9" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="F9" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="E9" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="F9" s="1" t="s">
-        <v>92</v>
-      </c>
       <c r="G9" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H9" s="1"/>
       <c r="I9" s="1"/>
       <c r="J9" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="K9" s="1"/>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="C10" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="B10" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>105</v>
-      </c>
       <c r="D10" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="F10" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="E10" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>92</v>
-      </c>
       <c r="G10" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H10" s="1"/>
       <c r="I10" s="1"/>
       <c r="J10" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="K10" s="1"/>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>7</v>
       </c>
@@ -2231,28 +2205,28 @@
         <v>7</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D11" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="F11" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="E11" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="F11" s="1" t="s">
-        <v>92</v>
-      </c>
       <c r="G11" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H11" s="1"/>
       <c r="I11" s="1"/>
       <c r="J11" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="K11" s="1"/>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>6</v>
       </c>
@@ -2260,28 +2234,28 @@
         <v>6</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D12" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="F12" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="E12" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>92</v>
-      </c>
       <c r="G12" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H12" s="1"/>
       <c r="I12" s="1"/>
       <c r="J12" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="K12" s="1"/>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>8</v>
       </c>
@@ -2289,28 +2263,28 @@
         <v>8</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D13" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="F13" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="E13" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="F13" s="1" t="s">
-        <v>92</v>
-      </c>
       <c r="G13" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H13" s="1"/>
       <c r="I13" s="1"/>
       <c r="J13" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="K13" s="1"/>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>9</v>
       </c>
@@ -2318,86 +2292,86 @@
         <v>9</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D14" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="F14" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="E14" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="F14" s="1" t="s">
-        <v>92</v>
-      </c>
       <c r="G14" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H14" s="1"/>
       <c r="I14" s="1"/>
       <c r="J14" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="K14" s="1"/>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B15" s="7" t="s">
         <v>26</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D15" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="F15" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="E15" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="F15" s="1" t="s">
+      <c r="G15" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="H15" s="1" t="s">
         <v>92</v>
-      </c>
-      <c r="G15" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="H15" s="1" t="s">
-        <v>93</v>
       </c>
       <c r="I15" s="1"/>
       <c r="J15" s="1"/>
       <c r="K15" s="1"/>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B16" s="7" t="s">
         <v>25</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D16" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="F16" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="E16" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="F16" s="1" t="s">
+      <c r="G16" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="H16" s="1" t="s">
         <v>92</v>
-      </c>
-      <c r="G16" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="H16" s="1" t="s">
-        <v>93</v>
       </c>
       <c r="I16" s="1"/>
       <c r="J16" s="1"/>
       <c r="K16" s="1"/>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>22</v>
       </c>
@@ -2405,457 +2379,457 @@
         <v>22</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D17" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="F17" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="E17" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="F17" s="1" t="s">
+      <c r="G17" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="H17" s="1" t="s">
         <v>92</v>
-      </c>
-      <c r="G17" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="H17" s="1" t="s">
-        <v>93</v>
       </c>
       <c r="I17" s="1"/>
       <c r="J17" s="1"/>
       <c r="K17" s="1"/>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
         <v>39</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D18" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="F18" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="E18" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="F18" s="1" t="s">
-        <v>92</v>
-      </c>
       <c r="G18" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H18" s="1"/>
       <c r="I18" s="1"/>
       <c r="J18" s="1"/>
       <c r="K18" s="1"/>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B19" s="7" t="s">
         <v>18</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D19" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="F19" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="E19" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="F19" s="1" t="s">
-        <v>92</v>
-      </c>
       <c r="G19" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H19" s="1"/>
       <c r="I19" s="1"/>
       <c r="J19" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="K19" s="1"/>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B20" s="1"/>
       <c r="C20" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="E20" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="D20" s="1" t="s">
+      <c r="F20" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="E20" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="F20" s="1" t="s">
-        <v>92</v>
-      </c>
       <c r="G20" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H20" s="1"/>
       <c r="I20" s="1"/>
       <c r="J20" s="1"/>
       <c r="K20" s="1"/>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B21" s="1"/>
       <c r="C21" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D21" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="F21" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="E21" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="F21" s="1" t="s">
-        <v>92</v>
-      </c>
       <c r="G21" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H21" s="1"/>
       <c r="I21" s="1"/>
       <c r="J21" s="1"/>
       <c r="K21" s="1"/>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B22" s="1"/>
       <c r="C22" s="1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D22" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="F22" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="E22" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="F22" s="1" t="s">
-        <v>92</v>
-      </c>
       <c r="G22" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H22" s="1"/>
       <c r="I22" s="1"/>
       <c r="J22" s="1"/>
       <c r="K22" s="1"/>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B23" s="1"/>
       <c r="C23" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F23" s="1"/>
       <c r="G23" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H23" s="1"/>
       <c r="I23" s="1"/>
       <c r="J23" s="1"/>
       <c r="K23" s="1"/>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B24" s="1"/>
       <c r="C24" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F24" s="1"/>
       <c r="G24" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="I24" s="1"/>
       <c r="J24" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="K24" s="1"/>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B25" s="1"/>
       <c r="C25" s="1">
         <v>2143543</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F25" s="1"/>
       <c r="G25" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H25" s="1"/>
       <c r="I25" s="1"/>
       <c r="J25" s="1"/>
       <c r="K25" s="1"/>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B26" s="1"/>
       <c r="C26" s="1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F26" s="1"/>
       <c r="G26" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H26" s="1"/>
       <c r="I26" s="1"/>
       <c r="J26" s="1"/>
       <c r="K26" s="1"/>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B27" s="1"/>
       <c r="C27" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F27" s="1"/>
       <c r="G27" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H27" s="1"/>
       <c r="I27" s="1"/>
       <c r="J27" s="1"/>
       <c r="K27" s="1"/>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B28" s="1"/>
       <c r="C28" s="1" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D28" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="F28" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="E28" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="F28" s="1" t="s">
-        <v>92</v>
-      </c>
       <c r="G28" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H28" s="1"/>
       <c r="I28" s="1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="J28" s="1"/>
       <c r="K28" s="1"/>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B29" s="7" t="s">
         <v>16</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D29" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="F29" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="E29" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="F29" s="1" t="s">
-        <v>92</v>
-      </c>
       <c r="G29" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H29" s="1"/>
       <c r="I29" s="1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="J29" s="1"/>
       <c r="K29" s="1"/>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B30" s="1"/>
       <c r="C30" s="1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D30" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="F30" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="E30" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="F30" s="1" t="s">
-        <v>92</v>
-      </c>
       <c r="G30" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H30" s="1"/>
       <c r="I30" s="1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="J30" s="1"/>
       <c r="K30" s="1"/>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B31" s="1"/>
       <c r="C31" s="1" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D31" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="F31" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="E31" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="F31" s="1" t="s">
-        <v>92</v>
-      </c>
       <c r="G31" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H31" s="1"/>
       <c r="I31" s="1"/>
       <c r="J31" s="1"/>
       <c r="K31" s="1"/>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B32" s="1"/>
       <c r="C32" s="1" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D32" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="F32" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="E32" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="F32" s="1" t="s">
-        <v>92</v>
-      </c>
       <c r="G32" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H32" s="1"/>
       <c r="I32" s="1"/>
       <c r="J32" s="1"/>
       <c r="K32" s="1"/>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B33" s="1"/>
       <c r="C33" s="1" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E33" s="1"/>
       <c r="F33" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G33" s="1"/>
       <c r="H33" s="1"/>
       <c r="I33" s="1"/>
       <c r="J33" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="K33" s="1"/>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B34" s="1"/>
       <c r="C34" s="1" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E34" s="1"/>
       <c r="F34" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G34" s="1"/>
       <c r="H34" s="1"/>
       <c r="I34" s="1"/>
       <c r="J34" s="1"/>
       <c r="K34" s="1" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.35">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
         <v>40</v>
       </c>
@@ -2863,53 +2837,53 @@
         <v>40</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F35" s="1"/>
       <c r="G35" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H35" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="I35" s="1"/>
       <c r="J35" s="1"/>
       <c r="K35" s="1"/>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F36" s="1"/>
       <c r="G36" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H36" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="I36" s="1"/>
       <c r="J36" s="1"/>
       <c r="K36" s="1"/>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
         <v>19</v>
       </c>
@@ -2917,130 +2891,130 @@
         <v>19</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D37" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="E37" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="F37" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="E37" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="F37" s="1" t="s">
-        <v>92</v>
-      </c>
       <c r="G37" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H37" s="1"/>
       <c r="I37" s="1"/>
       <c r="J37" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="K37" s="1" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.35">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B38" s="1"/>
       <c r="C38" s="1" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D38" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="F38" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="E38" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="F38" s="1" t="s">
-        <v>92</v>
-      </c>
       <c r="G38" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H38" s="1"/>
       <c r="I38" s="1"/>
       <c r="J38" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="K38" s="1" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.35">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A39" s="1" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B39" s="1"/>
       <c r="C39" s="1">
         <v>3265</v>
       </c>
       <c r="D39" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="E39" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="F39" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="E39" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="F39" s="1" t="s">
-        <v>92</v>
-      </c>
       <c r="G39" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H39" s="1"/>
       <c r="I39" s="1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="J39" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="K39" s="1" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.35">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B40" s="1"/>
       <c r="C40" s="1">
         <v>64000</v>
       </c>
       <c r="D40" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="E40" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="F40" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="E40" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="F40" s="1" t="s">
-        <v>92</v>
-      </c>
       <c r="G40" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H40" s="1"/>
       <c r="I40" s="1"/>
       <c r="J40" s="1"/>
       <c r="K40" s="1" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.35">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B41" s="1"/>
       <c r="C41" s="1" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E41" s="1"/>
       <c r="F41" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G41" s="1"/>
       <c r="H41" s="1"/>

</xml_diff>